<commit_message>
Updated positive end expiratory pressure outputs for both respiratory and mechanical ventilator system data.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CC94A9-6408-4CE2-B6A2-1A5B770A105E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7DDD18-EA03-4658-9421-72B7A7204BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26295" yWindow="5670" windowWidth="30945" windowHeight="24405" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28980" yWindow="4305" windowWidth="25425" windowHeight="23445" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="COPD" sheetId="13" r:id="rId3"/>
     <sheet name="Recruitment" sheetId="14" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -454,45 +454,6 @@
 }</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.6, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 13, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 9, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 20.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.42 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 35, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 17, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>StandardMale.json</t>
   </si>
   <si>
@@ -659,6 +620,45 @@
   "InspiratoryPressure": { "ScalarPressure": { "Value": 34, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 18, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.42 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 44, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 17, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.6, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 9, "Unit": "1/min" } }
   }}
 }</t>
   </si>
@@ -735,7 +735,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -773,11 +773,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -831,6 +868,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -842,14 +888,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1249,52 +1295,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="F2" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1306,11 +1352,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1329,72 +1375,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1406,13 +1452,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1422,13 +1468,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1436,15 +1482,15 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="B13" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H13" s="9"/>
     </row>
@@ -1452,13 +1498,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="B14" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1754,11 +1800,12 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1767,12 +1814,11 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1802,52 +1848,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="F2" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1859,11 +1905,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1882,72 +1928,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1955,17 +2001,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="27"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -1973,13 +2019,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -1989,13 +2035,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2005,13 +2051,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2019,15 +2065,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -2035,13 +2081,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2339,13 +2385,13 @@
       <c r="A29" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
       <c r="G29" s="1" t="s">
         <v>6</v>
       </c>
@@ -2357,13 +2403,13 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
       <c r="G30" s="9" t="s">
         <v>62</v>
       </c>
@@ -2373,15 +2419,15 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H31" s="9"/>
     </row>
@@ -2389,13 +2435,13 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
+      <c r="B32" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
     </row>
@@ -2693,13 +2739,13 @@
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="24" t="s">
+      <c r="B45" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
       <c r="G45" s="1" t="s">
         <v>6</v>
       </c>
@@ -2711,13 +2757,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
       <c r="G46" s="9" t="s">
         <v>78</v>
       </c>
@@ -2727,15 +2773,15 @@
       <c r="A47" s="8">
         <v>3</v>
       </c>
-      <c r="B47" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
+      <c r="B47" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
       <c r="G47" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H47" s="9"/>
     </row>
@@ -2743,13 +2789,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
+      <c r="B48" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
     </row>
@@ -3045,15 +3091,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3068,12 +3111,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B45:F45"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3102,52 +3148,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="F2" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3159,11 +3205,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3182,72 +3228,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3259,13 +3305,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3273,13 +3319,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3289,13 +3335,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3305,13 +3351,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3319,15 +3365,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>119</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="B15" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3335,13 +3381,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3385,7 +3431,7 @@
         <v>28</v>
       </c>
       <c r="E18" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>97</v>
@@ -3409,7 +3455,7 @@
         <v>28</v>
       </c>
       <c r="E19" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>96</v>
@@ -3433,7 +3479,7 @@
         <v>28</v>
       </c>
       <c r="E20" s="2">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="F20" s="11" t="s">
         <v>93</v>
@@ -3615,13 +3661,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3633,13 +3679,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="9" t="s">
         <v>79</v>
       </c>
@@ -3649,15 +3695,15 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
+      <c r="B30" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
       <c r="G30" s="9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3665,13 +3711,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="B31" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3715,7 +3761,7 @@
         <v>28</v>
       </c>
       <c r="E33" s="2">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>97</v>
@@ -3739,7 +3785,7 @@
         <v>28</v>
       </c>
       <c r="E34" s="2">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F34" s="11" t="s">
         <v>96</v>
@@ -3763,7 +3809,7 @@
         <v>28</v>
       </c>
       <c r="E35" s="2">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="F35" s="11" t="s">
         <v>93</v>
@@ -3945,13 +3991,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -3963,13 +4009,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
       <c r="G44" s="9" t="s">
         <v>80</v>
       </c>
@@ -3979,15 +4025,15 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
+      <c r="B45" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
       <c r="G45" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -3995,13 +4041,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
+      <c r="B46" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4045,7 +4091,7 @@
         <v>28</v>
       </c>
       <c r="E48" s="2">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F48" s="11" t="s">
         <v>97</v>
@@ -4069,7 +4115,7 @@
         <v>28</v>
       </c>
       <c r="E49" s="2">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="F49" s="11" t="s">
         <v>96</v>
@@ -4273,15 +4319,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4296,12 +4339,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4330,52 +4376,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="F2" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+        <v>119</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4387,11 +4433,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4410,72 +4456,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4483,17 +4529,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="27"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -4501,15 +4547,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="B12" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4517,13 +4563,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4533,13 +4579,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4547,15 +4593,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="B15" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4563,13 +4609,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4643,7 +4689,7 @@
         <v>70</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -4675,13 +4721,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4693,15 +4739,15 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="B22" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -4709,13 +4755,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="B23" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4837,7 +4883,7 @@
         <v>70</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -4915,6 +4961,20 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -4925,20 +4985,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Updates to mechanical ventilator validation.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7DDD18-EA03-4658-9421-72B7A7204BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793E69F9-E844-4BC5-9C10-E95623DDC71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28980" yWindow="4305" windowWidth="25425" windowHeight="23445" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26850" yWindow="3765" windowWidth="28425" windowHeight="24870" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -18,8 +18,19 @@
     <sheet name="COPD" sheetId="13" r:id="rId3"/>
     <sheet name="Recruitment" sheetId="14" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -426,32 +437,6 @@
   </si>
   <si>
     <t>[0.93, 0.98]</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.50 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.31 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 21, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 21, "Unit": "1/min" } }
-  }}
-}</t>
   </si>
   <si>
     <t>StandardMale.json</t>
@@ -585,19 +570,6 @@
 | PC-CMV | 520   | Adjust         | NA           | NA  | 0.87   | 23       | 18            | 0.5 |</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.80 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 25.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
   {
     "Severity": [ 
@@ -654,9 +626,48 @@
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
   "Mode": "ContinuousMandatoryVentilation", 
   "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.31 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 21.5, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 21, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.80 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 26, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.50 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 24.7, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.6, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 15.5, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 9, "Unit": "1/min" } }
   }}
@@ -868,15 +879,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -887,6 +889,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1295,52 +1306,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1352,11 +1363,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1375,72 +1386,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1452,13 +1463,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1468,13 +1479,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1482,15 +1493,15 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="B13" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H13" s="9"/>
     </row>
@@ -1498,13 +1509,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="B14" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1800,12 +1811,11 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1814,11 +1824,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1848,52 +1859,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1905,11 +1916,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1928,72 +1939,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2019,13 +2030,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2035,13 +2046,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2051,13 +2062,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2065,15 +2076,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -2081,13 +2092,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2385,13 +2396,13 @@
       <c r="A29" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
       <c r="G29" s="1" t="s">
         <v>6</v>
       </c>
@@ -2403,13 +2414,13 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
       <c r="G30" s="9" t="s">
         <v>62</v>
       </c>
@@ -2419,15 +2430,15 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="B31" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H31" s="9"/>
     </row>
@@ -2435,13 +2446,13 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
+      <c r="B32" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
     </row>
@@ -2739,13 +2750,13 @@
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="18" t="s">
+      <c r="B45" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="18"/>
+      <c r="C45" s="24"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
       <c r="G45" s="1" t="s">
         <v>6</v>
       </c>
@@ -2757,13 +2768,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="B46" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
       <c r="G46" s="9" t="s">
         <v>78</v>
       </c>
@@ -2773,15 +2784,15 @@
       <c r="A47" s="8">
         <v>3</v>
       </c>
-      <c r="B47" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
+      <c r="B47" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
       <c r="G47" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H47" s="9"/>
     </row>
@@ -2789,13 +2800,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-      <c r="F48" s="19"/>
+      <c r="B48" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
     </row>
@@ -3091,12 +3102,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B45:F45"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3111,15 +3125,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3148,52 +3159,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>123</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3205,11 +3216,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3228,72 +3239,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3305,13 +3316,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3319,13 +3330,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3335,13 +3346,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3351,13 +3362,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3365,15 +3376,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3381,13 +3392,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3503,7 +3514,7 @@
         <v>28</v>
       </c>
       <c r="E21" s="2">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>98</v>
@@ -3661,13 +3672,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3679,13 +3690,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="9" t="s">
         <v>79</v>
       </c>
@@ -3695,15 +3706,15 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
+      <c r="B30" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
       <c r="G30" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3711,13 +3722,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="B31" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3833,7 +3844,7 @@
         <v>28</v>
       </c>
       <c r="E36" s="2">
-        <v>0.49</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F36" s="11" t="s">
         <v>98</v>
@@ -3991,13 +4002,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4009,13 +4020,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
       <c r="G44" s="9" t="s">
         <v>80</v>
       </c>
@@ -4025,15 +4036,15 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
+      <c r="B45" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
       <c r="G45" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -4041,13 +4052,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
+      <c r="B46" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4163,7 +4174,7 @@
         <v>28</v>
       </c>
       <c r="E51" s="2">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="F51" s="11" t="s">
         <v>98</v>
@@ -4319,12 +4330,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4339,15 +4353,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4376,52 +4387,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+        <v>117</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4433,11 +4444,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4456,72 +4467,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4547,15 +4558,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="B12" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4563,13 +4574,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4579,13 +4590,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4593,15 +4604,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4609,13 +4620,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4689,7 +4700,7 @@
         <v>70</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -4721,13 +4732,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4739,15 +4750,15 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
+      <c r="B22" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
       <c r="G22" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -4755,13 +4766,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="B23" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4883,7 +4894,7 @@
         <v>70</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -4961,20 +4972,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -4985,6 +4982,20 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated CO2 binding bounds to better meet validation. Put alveoli diffusion area modification action and condition back in. Tweaked ARDS shunt mapping.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793E69F9-E844-4BC5-9C10-E95623DDC71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3A3869-4224-4D78-B625-3DEA43EE99AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26850" yWindow="3765" windowWidth="28425" windowHeight="24870" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27765" yWindow="4920" windowWidth="28230" windowHeight="26025" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="150">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -672,6 +672,21 @@
   "RespirationRate": { "ScalarFrequency": { "Value": 9, "Unit": "1/min" } }
   }}
 }</t>
+  </si>
+  <si>
+    <t>[200, 300]</t>
+  </si>
+  <si>
+    <t>ferguson2012berlin</t>
+  </si>
+  <si>
+    <t>[100, 200]</t>
+  </si>
+  <si>
+    <t>lessThanValue</t>
+  </si>
+  <si>
+    <t>greaterThanValue</t>
   </si>
 </sst>
 </file>
@@ -879,6 +894,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -889,15 +913,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1290,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{415C2FCE-0151-4310-828D-F5A5D79BC461}">
-  <dimension ref="A1:AMJ26"/>
+  <dimension ref="A1:AMJ27"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="12" customWidth="1"/>
@@ -1306,52 +1321,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1363,11 +1378,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1386,72 +1401,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1463,13 +1478,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1479,13 +1494,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1493,13 +1508,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
         <v>122</v>
       </c>
@@ -1509,13 +1524,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1809,13 +1824,38 @@
       </c>
       <c r="H26" s="10"/>
     </row>
+    <row r="27" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E27" s="2">
+        <v>300</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" s="10"/>
+    </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1824,12 +1864,11 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1843,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B553321-70FB-4CC9-8C9D-15BA9D08D273}">
-  <dimension ref="A1:AMJ60"/>
+  <dimension ref="A1:AMJ63"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="12" customWidth="1"/>
@@ -1859,52 +1898,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1916,11 +1955,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1939,72 +1978,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2030,13 +2069,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2046,13 +2085,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2062,13 +2101,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2076,13 +2115,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>123</v>
       </c>
@@ -2092,13 +2131,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2392,126 +2431,126 @@
       </c>
       <c r="H28" s="10"/>
     </row>
-    <row r="29" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H29" s="10"/>
+    </row>
+    <row r="30" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B30" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="1" t="s">
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H29" s="15" t="s">
+      <c r="H30" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="8">
-        <v>2</v>
-      </c>
-      <c r="B30" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="H30" s="9"/>
-    </row>
-    <row r="31" spans="1:8" ht="187.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="B31" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="H31" s="9"/>
     </row>
-    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="187.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="8">
+        <v>2</v>
+      </c>
+      <c r="B33" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B34" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C34" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H33" s="15" t="s">
+      <c r="H34" s="15" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E34" s="2">
-        <v>12</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>37</v>
@@ -2526,7 +2565,7 @@
         <v>92</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H35" s="10"/>
     </row>
@@ -2535,22 +2574,22 @@
         <v>25</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E36" s="2">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H36" s="10"/>
     </row>
@@ -2559,22 +2598,22 @@
         <v>25</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E37" s="2">
-        <v>0.56999999999999995</v>
+        <v>35</v>
       </c>
       <c r="F37" s="11" t="s">
         <v>93</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="H37" s="10"/>
     </row>
@@ -2583,7 +2622,7 @@
         <v>25</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>27</v>
@@ -2592,85 +2631,85 @@
         <v>28</v>
       </c>
       <c r="E38" s="2">
-        <v>0.39</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="F38" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>83</v>
+      <c r="G38" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E39" s="2">
+        <v>0.39</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" s="2">
         <v>396</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H39" s="10"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="F40" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G40" s="13" t="s">
-        <v>46</v>
+      <c r="G40" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="H40" s="10"/>
     </row>
-    <row r="41" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F41" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>48</v>
+      <c r="G41" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="H41" s="10"/>
     </row>
@@ -2679,7 +2718,7 @@
         <v>29</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>31</v>
@@ -2688,37 +2727,37 @@
         <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F42" s="11" t="s">
         <v>92</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H43" s="10"/>
     </row>
@@ -2727,184 +2766,184 @@
         <v>25</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F44" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F44" s="11" t="s">
+      <c r="F45" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H44" s="10"/>
-    </row>
-    <row r="45" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F46" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="24" t="s">
+      <c r="B47" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="1" t="s">
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="15" t="s">
+      <c r="H47" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="8">
-        <v>3</v>
-      </c>
-      <c r="B46" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="H46" s="9"/>
-    </row>
-    <row r="47" spans="1:8" ht="187.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="8">
-        <v>3</v>
-      </c>
-      <c r="B47" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="H47" s="9"/>
-    </row>
-    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H48" s="9"/>
+    </row>
+    <row r="49" spans="1:8" ht="187.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="8">
+        <v>3</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="8">
+        <v>3</v>
+      </c>
+      <c r="B50" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="9"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B51" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C51" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F51" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G49" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H49" s="15" t="s">
+      <c r="H51" s="15" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E50" s="2">
-        <v>12</v>
-      </c>
-      <c r="F50" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G50" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="H50" s="10"/>
-    </row>
-    <row r="51" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E51" s="2">
-        <v>12</v>
-      </c>
-      <c r="F51" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G51" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="H51" s="10"/>
     </row>
     <row r="52" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E52" s="2">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H52" s="10"/>
     </row>
@@ -2913,22 +2952,22 @@
         <v>25</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E53" s="2">
-        <v>0.65</v>
+        <v>12</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G53" s="13" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="H53" s="10"/>
     </row>
@@ -2937,151 +2976,151 @@
         <v>25</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E54" s="2">
-        <v>0.61</v>
+        <v>33</v>
       </c>
       <c r="F54" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G54" s="2" t="s">
-        <v>83</v>
+      <c r="G54" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E55" s="2">
-        <v>396</v>
+        <v>0.65</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>66</v>
+        <v>93</v>
+      </c>
+      <c r="G55" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="H55" s="10"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>109</v>
+        <v>28</v>
+      </c>
+      <c r="E56" s="2">
+        <v>0.61</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G56" s="13" t="s">
-        <v>46</v>
+        <v>93</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>110</v>
+        <v>28</v>
+      </c>
+      <c r="E57" s="2">
+        <v>396</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>92</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="H57" s="10"/>
     </row>
-    <row r="58" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G58" s="2" t="s">
-        <v>47</v>
+      <c r="G58" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H59" s="10"/>
     </row>
     <row r="60" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>31</v>
@@ -3090,27 +3129,96 @@
         <v>55</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>92</v>
       </c>
       <c r="G60" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H60" s="10"/>
+    </row>
+    <row r="61" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H61" s="10"/>
+    </row>
+    <row r="62" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G62" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H60" s="10"/>
+      <c r="H62" s="10"/>
+    </row>
+    <row r="63" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E63" s="2">
+        <v>200</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H63" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3125,12 +3233,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3159,52 +3270,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3216,11 +3327,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3239,72 +3350,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3316,13 +3427,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3330,13 +3441,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3346,13 +3457,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3362,13 +3473,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3376,13 +3487,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>124</v>
       </c>
@@ -3392,13 +3503,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3672,13 +3783,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3690,13 +3801,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="9" t="s">
         <v>79</v>
       </c>
@@ -3706,13 +3817,13 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
       <c r="G30" s="9" t="s">
         <v>127</v>
       </c>
@@ -3722,13 +3833,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -4002,13 +4113,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4020,13 +4131,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
       <c r="G44" s="9" t="s">
         <v>80</v>
       </c>
@@ -4036,13 +4147,13 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="22" t="s">
+      <c r="B45" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
       <c r="G45" s="9" t="s">
         <v>128</v>
       </c>
@@ -4052,13 +4163,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4330,15 +4441,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4353,12 +4461,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4387,52 +4498,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4444,11 +4555,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4467,72 +4578,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4558,13 +4669,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>137</v>
       </c>
@@ -4574,13 +4685,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4590,13 +4701,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4604,13 +4715,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>129</v>
       </c>
@@ -4620,13 +4731,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4732,13 +4843,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4750,13 +4861,13 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="9" t="s">
         <v>135</v>
       </c>
@@ -4766,13 +4877,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4972,6 +5083,20 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -4982,20 +5107,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Update respiratory injury validation and calibration.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3A3869-4224-4D78-B625-3DEA43EE99AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AC6CE2-3EDD-4FA5-BB7A-B723377E680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27765" yWindow="4920" windowWidth="28230" windowHeight="26025" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29100" yWindow="5325" windowWidth="28230" windowHeight="25455" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -486,13 +486,6 @@
 | PC-CMV | 414   | Adjust         | NA           | 0.83  | 1.3   | 21       | 10            | 0.31 |</t>
   </si>
   <si>
-    <t>Ventilator settings are (VT Target = 7.3 mL/kg (ideal)):
-&lt;br /&gt;
-| Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| PC-CMV | 438   | Adjust         | NA           | 0.32  | 1.6   | 9       | 5            | 0.28 |</t>
-  </si>
-  <si>
     <t>Ventilator settings are (VT Target = 6.6 mL/kg (ideal)):
 &lt;br /&gt;
 | Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
@@ -512,13 +505,6 @@
 | Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
 | PC-CMV | 534   | Adjust         | NA           | 0.43  | 1.3   | 14       | 7            | 0.32 |</t>
-  </si>
-  <si>
-    <t>Ventilator settings are (VT Target = 10.9 mL/kg (ideal)):
-&lt;br /&gt;
-| Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| PC-CMV | 654   | Adjust         | NA           | 0.5  | 1.2   | 17       | 10            | 0.42 |</t>
   </si>
   <si>
     <t>Ventilator settings are set for TV = 6.9 mL/kg (ideal) and I:E = 0.5:
@@ -600,13 +586,55 @@
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
   "Mode": "ContinuousMandatoryVentilation", 
   "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.31 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 21.5, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 21, "Unit": "1/min" } }
   }}
 }</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.50 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 24.7, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>[200, 300]</t>
+  </si>
+  <si>
+    <t>ferguson2012berlin</t>
+  </si>
+  <si>
+    <t>[100, 200]</t>
+  </si>
+  <si>
+    <t>lessThanValue</t>
+  </si>
+  <si>
+    <t>greaterThanValue</t>
+  </si>
+  <si>
+    <t>Ventilator settings are (VT Target = 10.0 mL/kg (ideal)):
+&lt;br /&gt;
+| Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| PC-CMV | 600   | Adjust         | NA           | 0.5  | 1.1   | 16       | 10            | 0.42 |</t>
+  </si>
+  <si>
+    <t>Ventilator settings are (VT Target = 7.3 mL/kg (ideal)):
+&lt;br /&gt;
+| Mode   | VT (mL) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| PC-CMV | 438   | Adjust         | NA           | 0.32  | 1.2   | 12       | 5            | 0.32 |</t>
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
@@ -614,8 +642,8 @@
   "Mode": "ContinuousMandatoryVentilation", 
   "InspirationWaveform": "Square",
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.42 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 44, "Unit": "cmH2O" } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.1, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 42.5, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 17, "Unit": "1/min" } }
   }}
@@ -626,11 +654,24 @@
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
   "Mode": "ContinuousMandatoryVentilation", 
   "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.31 } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 14.5, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 12, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 21.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 21, "Unit": "1/min" } }
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 23.5, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
   }}
 }</t>
   </si>
@@ -646,47 +687,6 @@
   "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } }
   }}
 }</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.50 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 24.7, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.6, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 15.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 9, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>[200, 300]</t>
-  </si>
-  <si>
-    <t>ferguson2012berlin</t>
-  </si>
-  <si>
-    <t>[100, 200]</t>
-  </si>
-  <si>
-    <t>lessThanValue</t>
-  </si>
-  <si>
-    <t>greaterThanValue</t>
   </si>
 </sst>
 </file>
@@ -1509,7 +1509,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -1835,13 +1835,13 @@
         <v>31</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E27" s="2">
         <v>300</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>91</v>
@@ -2116,7 +2116,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -2277,7 +2277,7 @@
         <v>28</v>
       </c>
       <c r="E22" s="2">
-        <v>0.31</v>
+        <v>0.2</v>
       </c>
       <c r="F22" s="11" t="s">
         <v>93</v>
@@ -2445,10 +2445,10 @@
         <v>55</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>91</v>
@@ -2494,14 +2494,14 @@
         <v>2</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
       <c r="E32" s="19"/>
       <c r="F32" s="19"/>
       <c r="G32" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H32" s="9"/>
     </row>
@@ -2655,7 +2655,7 @@
         <v>28</v>
       </c>
       <c r="E39" s="2">
-        <v>0.39</v>
+        <v>0.3</v>
       </c>
       <c r="F39" s="11" t="s">
         <v>93</v>
@@ -2823,10 +2823,10 @@
         <v>55</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>91</v>
@@ -2872,14 +2872,14 @@
         <v>3</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C49" s="19"/>
       <c r="D49" s="19"/>
       <c r="E49" s="19"/>
       <c r="F49" s="19"/>
       <c r="G49" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H49" s="9"/>
     </row>
@@ -3033,7 +3033,7 @@
         <v>28</v>
       </c>
       <c r="E56" s="2">
-        <v>0.61</v>
+        <v>0.4</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>93</v>
@@ -3198,13 +3198,13 @@
         <v>31</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E63" s="2">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>91</v>
@@ -3488,14 +3488,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
       <c r="E15" s="19"/>
       <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3601,7 +3601,7 @@
         <v>28</v>
       </c>
       <c r="E20" s="2">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F20" s="11" t="s">
         <v>93</v>
@@ -3818,14 +3818,14 @@
         <v>2</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>
       <c r="F30" s="19"/>
       <c r="G30" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3931,7 +3931,7 @@
         <v>28</v>
       </c>
       <c r="E35" s="2">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F35" s="11" t="s">
         <v>93</v>
@@ -4148,14 +4148,14 @@
         <v>3</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="19"/>
       <c r="E45" s="19"/>
       <c r="F45" s="19"/>
       <c r="G45" s="9" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -4309,7 +4309,7 @@
         <v>28</v>
       </c>
       <c r="E52" s="2">
-        <v>0.48</v>
+        <v>0.25</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>99</v>
@@ -4333,7 +4333,7 @@
         <v>28</v>
       </c>
       <c r="E53" s="2">
-        <v>654</v>
+        <v>600</v>
       </c>
       <c r="F53" s="11" t="s">
         <v>92</v>
@@ -4528,7 +4528,7 @@
         <v>117</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G2" s="24"/>
       <c r="H2" s="24"/>
@@ -4670,14 +4670,14 @@
         <v>1</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
       <c r="E12" s="19"/>
       <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4716,14 +4716,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
       <c r="E15" s="19"/>
       <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4811,7 +4811,7 @@
         <v>70</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -4862,14 +4862,14 @@
         <v>2</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
       <c r="G22" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -5005,7 +5005,7 @@
         <v>70</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H28" s="10"/>
     </row>

</xml_diff>

<commit_message>
Add respiratory disease diffusion effects back in and calibrated.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AC6CE2-3EDD-4FA5-BB7A-B723377E680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FCC6CA-EB35-48E4-8FF8-A1018F64529F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29100" yWindow="5325" windowWidth="28230" windowHeight="25455" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25740" yWindow="2850" windowWidth="28230" windowHeight="25455" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="148">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -346,21 +346,6 @@
     <t>QS/QT (0.22 +/- 0.14)</t>
   </si>
   <si>
-    <t>[35, 39]</t>
-  </si>
-  <si>
-    <t>[81, 97]</t>
-  </si>
-  <si>
-    <t>[0.96, 0.98]</t>
-  </si>
-  <si>
-    <t>[7.33, 7.43]</t>
-  </si>
-  <si>
-    <t>[312, 373]</t>
-  </si>
-  <si>
     <t>PaO2/FiO2</t>
   </si>
   <si>
@@ -370,9 +355,6 @@
     <t>maj2023ventilatory</t>
   </si>
   <si>
-    <t>Chatburn2011</t>
-  </si>
-  <si>
     <t>gadrey2019imputation</t>
   </si>
   <si>
@@ -443,15 +425,6 @@
   </si>
   <si>
     <t>{ "AdvanceUntilStable":  {} }</t>
-  </si>
-  <si>
-    <t>A healthy male patient with a predicted body weight of 60 kg is mechanically ventilated.  No single reference provides enough data to link severity of disease to ventilator settings and expected values for gas exchange and mechanics. Several references were combined for a complete set of simulation parameters. These are the data sources:
- - Resistance: Inspiratory resistance (Rinsp) is assumed equal to expiratory resistance (Rexp), taken from Arnal et al @cite arnal2018parameters Table 9.
- - Compliance: Taken from Maj et al @cite maj2023ventilatory Table 1 derived as tidal volume (i.e., mL/kg x PBW calculated) divided by driving pressure. 
- - Dead space:  Taken from the Chatburn et al Handbook for Respiratory Care @cite Chatburn2011.
- - Shunt:  Taken from the Chatburn et al Handbook for Respiratory Care @cite Chatburn2011.
- - Ventilator Settings: Taken from Arnal et al @cite arnal2018parameters Table 2 for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et al @cite arnal2018parameters for passive patients. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
- - Blood Gas Values: Taken from Arnal et al @cite arnal2018parameters Table 2. Expected values for SpO2 were calculated from PaO2 using the equation from Gadrey et al @cite gadrey2019imputation.</t>
   </si>
   <si>
     <t>A male patient with a predicted body weight of 60 kg is mechanically ventilated with varying severities of ARDS.  No single reference provides enough data to link severity of disease to ventilator settings and expected values for gas exchange and mechanics. Several references were combined for a complete set of simulation parameters. These are the data sources:
@@ -687,6 +660,27 @@
   "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } }
   }}
 }</t>
+  </si>
+  <si>
+    <t>[0.2, 0.4]</t>
+  </si>
+  <si>
+    <t>kacmarek2016egan</t>
+  </si>
+  <si>
+    <t>[400, 500]</t>
+  </si>
+  <si>
+    <t>[7.35, 7.45]</t>
+  </si>
+  <si>
+    <t>A healthy male patient with a predicted body weight of 60 kg is mechanically ventilated.  No single reference provides enough data to link severity of disease to ventilator settings and expected values for gas exchange and mechanics. Several references were combined for a complete set of simulation parameters. These are the data sources:
+ - Resistance: Inspiratory resistance (Rinsp) is assumed equal to expiratory resistance (Rexp), taken from Arnal et al @cite arnal2018parameters Table 9.
+ - Compliance: Taken from Maj et al @cite maj2023ventilatory Table 1 derived as tidal volume (i.e., mL/kg x PBW calculated) divided by driving pressure. 
+ - Dead space:  Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.
+ - Shunt:  Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.
+ - Ventilator Settings: Taken from Arnal et al @cite arnal2018parameters Table 2 for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et al @cite arnal2018parameters for passive patients. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
+ - Blood Gas Values: Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.</t>
   </si>
 </sst>
 </file>
@@ -894,15 +888,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -913,6 +898,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1321,52 +1315,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>119</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1378,11 +1372,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1401,72 +1395,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1478,13 +1472,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1494,13 +1488,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1508,15 +1502,15 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="B13" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="H13" s="9"/>
     </row>
@@ -1524,13 +1518,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="B14" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1577,7 +1571,7 @@
         <v>10</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>42</v>
@@ -1601,7 +1595,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>43</v>
@@ -1625,7 +1619,7 @@
         <v>54</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>44</v>
@@ -1643,13 +1637,13 @@
         <v>27</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0.25</v>
+        <v>55</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>77</v>
@@ -1667,13 +1661,13 @@
         <v>27</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>28</v>
+        <v>135</v>
       </c>
       <c r="E20" s="2">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>83</v>
@@ -1697,7 +1691,7 @@
         <v>444</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>66</v>
@@ -1718,10 +1712,10 @@
         <v>55</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>89</v>
+        <v>146</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>46</v>
@@ -1739,13 +1733,13 @@
         <v>31</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>87</v>
+        <v>136</v>
+      </c>
+      <c r="E23" s="2">
+        <v>75</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>48</v>
@@ -1763,13 +1757,13 @@
         <v>31</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>86</v>
+        <v>135</v>
+      </c>
+      <c r="E24" s="2">
+        <v>45</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>47</v>
@@ -1787,13 +1781,13 @@
         <v>27</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>88</v>
+        <v>136</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0.95</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>95</v>
+        <v>144</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>49</v>
@@ -1814,13 +1808,13 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H26" s="10"/>
     </row>
@@ -1835,27 +1829,26 @@
         <v>31</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E27" s="2">
         <v>300</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H27" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1864,11 +1857,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1898,52 +1892,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>120</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1955,11 +1949,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1978,72 +1972,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2069,13 +2063,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2085,13 +2079,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2101,13 +2095,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2115,15 +2109,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -2131,13 +2125,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2184,7 +2178,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>42</v>
@@ -2208,7 +2202,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>43</v>
@@ -2232,7 +2226,7 @@
         <v>40</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>44</v>
@@ -2256,7 +2250,7 @@
         <v>0.54</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>77</v>
@@ -2280,7 +2274,7 @@
         <v>0.2</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>83</v>
@@ -2304,7 +2298,7 @@
         <v>414</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>66</v>
@@ -2325,10 +2319,10 @@
         <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>46</v>
@@ -2349,10 +2343,10 @@
         <v>55</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>48</v>
@@ -2373,10 +2367,10 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>47</v>
@@ -2397,10 +2391,10 @@
         <v>55</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>49</v>
@@ -2421,13 +2415,13 @@
         <v>55</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -2445,13 +2439,13 @@
         <v>55</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -2459,13 +2453,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2477,13 +2471,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2493,15 +2487,15 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
+      <c r="B32" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
       <c r="G32" s="9" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="H32" s="9"/>
     </row>
@@ -2509,13 +2503,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
+      <c r="B33" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2562,7 +2556,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>42</v>
@@ -2586,7 +2580,7 @@
         <v>12</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>43</v>
@@ -2610,7 +2604,7 @@
         <v>35</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>44</v>
@@ -2634,7 +2628,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G38" s="13" t="s">
         <v>77</v>
@@ -2658,7 +2652,7 @@
         <v>0.3</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>83</v>
@@ -2682,7 +2676,7 @@
         <v>396</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>66</v>
@@ -2703,10 +2697,10 @@
         <v>55</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>46</v>
@@ -2727,10 +2721,10 @@
         <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>48</v>
@@ -2751,10 +2745,10 @@
         <v>55</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>47</v>
@@ -2775,10 +2769,10 @@
         <v>55</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>49</v>
@@ -2799,13 +2793,13 @@
         <v>55</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H45" s="10"/>
     </row>
@@ -2823,13 +2817,13 @@
         <v>55</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H46" s="10"/>
     </row>
@@ -2837,13 +2831,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="18"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2855,13 +2849,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="19" t="s">
+      <c r="B48" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-      <c r="F48" s="19"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
       <c r="G48" s="9" t="s">
         <v>78</v>
       </c>
@@ -2871,15 +2865,15 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
+      <c r="B49" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
       <c r="G49" s="9" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="H49" s="9"/>
     </row>
@@ -2887,13 +2881,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
+      <c r="B50" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -2940,7 +2934,7 @@
         <v>12</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G52" s="13" t="s">
         <v>42</v>
@@ -2964,7 +2958,7 @@
         <v>12</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G53" s="13" t="s">
         <v>43</v>
@@ -2988,7 +2982,7 @@
         <v>33</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>44</v>
@@ -3012,7 +3006,7 @@
         <v>0.65</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G55" s="13" t="s">
         <v>77</v>
@@ -3036,7 +3030,7 @@
         <v>0.4</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>83</v>
@@ -3060,7 +3054,7 @@
         <v>396</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>66</v>
@@ -3081,10 +3075,10 @@
         <v>55</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G58" s="13" t="s">
         <v>46</v>
@@ -3105,10 +3099,10 @@
         <v>55</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>48</v>
@@ -3129,10 +3123,10 @@
         <v>55</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>47</v>
@@ -3153,10 +3147,10 @@
         <v>55</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>49</v>
@@ -3177,13 +3171,13 @@
         <v>55</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H62" s="10"/>
     </row>
@@ -3198,27 +3192,30 @@
         <v>31</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="E63" s="2">
         <v>100</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H63" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3233,15 +3230,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3270,52 +3264,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3327,11 +3321,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3350,72 +3344,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3427,13 +3421,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3441,13 +3435,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3457,13 +3451,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3473,13 +3467,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3487,15 +3481,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3503,13 +3497,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3556,7 +3550,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>42</v>
@@ -3580,7 +3574,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>43</v>
@@ -3604,7 +3598,7 @@
         <v>60</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>44</v>
@@ -3625,10 +3619,10 @@
         <v>28</v>
       </c>
       <c r="E21" s="2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>77</v>
@@ -3652,7 +3646,7 @@
         <v>0.12</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>83</v>
@@ -3676,7 +3670,7 @@
         <v>438</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>66</v>
@@ -3697,10 +3691,10 @@
         <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>46</v>
@@ -3721,10 +3715,10 @@
         <v>55</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>48</v>
@@ -3748,7 +3742,7 @@
         <v>81</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>47</v>
@@ -3769,10 +3763,10 @@
         <v>55</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>49</v>
@@ -3783,13 +3777,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3801,13 +3795,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="9" t="s">
         <v>79</v>
       </c>
@@ -3817,15 +3811,15 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
+      <c r="B30" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
       <c r="G30" s="9" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3833,13 +3827,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="B31" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3886,7 +3880,7 @@
         <v>21</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>42</v>
@@ -3910,7 +3904,7 @@
         <v>33</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>43</v>
@@ -3934,7 +3928,7 @@
         <v>68</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>44</v>
@@ -3955,10 +3949,10 @@
         <v>28</v>
       </c>
       <c r="E36" s="2">
-        <v>0.55000000000000004</v>
+        <v>0.49</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>77</v>
@@ -3982,7 +3976,7 @@
         <v>0.19</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>83</v>
@@ -4006,7 +4000,7 @@
         <v>534</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>66</v>
@@ -4027,10 +4021,10 @@
         <v>55</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>46</v>
@@ -4051,10 +4045,10 @@
         <v>55</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>48</v>
@@ -4078,7 +4072,7 @@
         <v>81</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>47</v>
@@ -4099,10 +4093,10 @@
         <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>49</v>
@@ -4113,13 +4107,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4131,13 +4125,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
       <c r="G44" s="9" t="s">
         <v>80</v>
       </c>
@@ -4147,15 +4141,15 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
+      <c r="B45" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
       <c r="G45" s="9" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -4163,13 +4157,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
+      <c r="B46" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4216,7 +4210,7 @@
         <v>33</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G48" s="13" t="s">
         <v>42</v>
@@ -4240,7 +4234,7 @@
         <v>51</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G49" s="13" t="s">
         <v>43</v>
@@ -4264,7 +4258,7 @@
         <v>75</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G50" s="13" t="s">
         <v>44</v>
@@ -4285,10 +4279,10 @@
         <v>28</v>
       </c>
       <c r="E51" s="2">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G51" s="13" t="s">
         <v>77</v>
@@ -4312,7 +4306,7 @@
         <v>0.25</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>83</v>
@@ -4336,7 +4330,7 @@
         <v>600</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>66</v>
@@ -4357,10 +4351,10 @@
         <v>55</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>46</v>
@@ -4381,10 +4375,10 @@
         <v>55</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>48</v>
@@ -4408,7 +4402,7 @@
         <v>81</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>47</v>
@@ -4429,10 +4423,10 @@
         <v>55</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>49</v>
@@ -4441,12 +4435,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4461,15 +4458,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4498,52 +4492,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>130</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+        <v>111</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4555,11 +4549,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4578,72 +4572,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4669,15 +4663,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="B12" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4685,13 +4679,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4701,13 +4695,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4715,15 +4709,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4731,13 +4725,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="B16" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4811,7 +4805,7 @@
         <v>70</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -4843,13 +4837,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4861,15 +4855,15 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
+      <c r="B22" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
       <c r="G22" s="9" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -4877,13 +4871,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="B23" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -5005,7 +4999,7 @@
         <v>70</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -5029,7 +5023,7 @@
         <v>70</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -5083,20 +5077,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -5107,6 +5087,20 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Ventilator triggering and validation updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FCC6CA-EB35-48E4-8FF8-A1018F64529F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55A49B3-CCC5-4E90-BE65-13CB8D2EA46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25740" yWindow="2850" windowWidth="28230" windowHeight="25455" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25710" yWindow="2040" windowWidth="29130" windowHeight="27735" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -276,9 +276,6 @@
     }</t>
   </si>
   <si>
-    <t>VT (set)</t>
-  </si>
-  <si>
     <t>MechanicalVentilatorRecruitment</t>
   </si>
   <si>
@@ -681,6 +678,9 @@
  - Shunt:  Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.
  - Ventilator Settings: Taken from Arnal et al @cite arnal2018parameters Table 2 for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et al @cite arnal2018parameters for passive patients. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
  - Blood Gas Values: Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.</t>
+  </si>
+  <si>
+    <t>VT (measured)</t>
   </si>
 </sst>
 </file>
@@ -888,6 +888,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -898,15 +907,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1315,52 +1315,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+        <v>81</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1372,11 +1372,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1395,72 +1395,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1472,13 +1472,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1488,13 +1488,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1502,15 +1502,15 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="B13" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H13" s="9"/>
     </row>
@@ -1518,13 +1518,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="B14" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1571,7 +1571,7 @@
         <v>10</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>42</v>
@@ -1595,7 +1595,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>43</v>
@@ -1619,7 +1619,7 @@
         <v>54</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>44</v>
@@ -1631,7 +1631,7 @@
         <v>25</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>27</v>
@@ -1640,13 +1640,13 @@
         <v>55</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F19" s="11" t="s">
-        <v>144</v>
-      </c>
       <c r="G19" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -1661,16 +1661,16 @@
         <v>27</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E20" s="2">
         <v>0.05</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H20" s="10"/>
     </row>
@@ -1691,10 +1691,10 @@
         <v>444</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H21" s="10"/>
     </row>
@@ -1712,10 +1712,10 @@
         <v>55</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>46</v>
@@ -1733,13 +1733,13 @@
         <v>31</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E23" s="2">
         <v>75</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>48</v>
@@ -1757,13 +1757,13 @@
         <v>31</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E24" s="2">
         <v>45</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>47</v>
@@ -1781,13 +1781,13 @@
         <v>27</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E25" s="2">
         <v>0.95</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>49</v>
@@ -1808,13 +1808,13 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H26" s="10"/>
     </row>
@@ -1829,26 +1829,27 @@
         <v>31</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E27" s="2">
         <v>300</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H27" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1857,12 +1858,11 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1892,52 +1892,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+        <v>81</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1949,11 +1949,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1972,72 +1972,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2063,13 +2063,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2079,13 +2079,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2095,13 +2095,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2109,15 +2109,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="B15" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -2125,13 +2125,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2178,7 +2178,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>42</v>
@@ -2202,7 +2202,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>43</v>
@@ -2226,7 +2226,7 @@
         <v>40</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>44</v>
@@ -2238,7 +2238,7 @@
         <v>25</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>27</v>
@@ -2250,10 +2250,10 @@
         <v>0.54</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H21" s="10"/>
     </row>
@@ -2274,10 +2274,10 @@
         <v>0.2</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H22" s="10"/>
     </row>
@@ -2298,10 +2298,10 @@
         <v>414</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H23" s="10"/>
     </row>
@@ -2319,10 +2319,10 @@
         <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>46</v>
@@ -2343,10 +2343,10 @@
         <v>55</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>48</v>
@@ -2367,10 +2367,10 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>47</v>
@@ -2391,10 +2391,10 @@
         <v>55</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>49</v>
@@ -2415,13 +2415,13 @@
         <v>55</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -2439,13 +2439,13 @@
         <v>55</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F29" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="F29" s="11" t="s">
-        <v>133</v>
-      </c>
       <c r="G29" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -2453,13 +2453,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2471,13 +2471,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2487,15 +2487,15 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
+      <c r="B32" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
       <c r="G32" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H32" s="9"/>
     </row>
@@ -2503,13 +2503,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
+      <c r="B33" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2556,7 +2556,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>42</v>
@@ -2580,7 +2580,7 @@
         <v>12</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>43</v>
@@ -2604,7 +2604,7 @@
         <v>35</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>44</v>
@@ -2616,7 +2616,7 @@
         <v>25</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>27</v>
@@ -2628,10 +2628,10 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H38" s="10"/>
     </row>
@@ -2652,10 +2652,10 @@
         <v>0.3</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H39" s="10"/>
     </row>
@@ -2676,10 +2676,10 @@
         <v>396</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H40" s="10"/>
     </row>
@@ -2697,10 +2697,10 @@
         <v>55</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>46</v>
@@ -2721,10 +2721,10 @@
         <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>48</v>
@@ -2745,10 +2745,10 @@
         <v>55</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>47</v>
@@ -2769,10 +2769,10 @@
         <v>55</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>49</v>
@@ -2793,13 +2793,13 @@
         <v>55</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H45" s="10"/>
     </row>
@@ -2817,13 +2817,13 @@
         <v>55</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H46" s="10"/>
     </row>
@@ -2831,13 +2831,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2849,15 +2849,15 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
       <c r="G48" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H48" s="9"/>
     </row>
@@ -2865,15 +2865,15 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="C49" s="22"/>
-      <c r="D49" s="22"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
+      <c r="B49" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
       <c r="G49" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H49" s="9"/>
     </row>
@@ -2881,13 +2881,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" s="22"/>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
+      <c r="B50" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -2934,7 +2934,7 @@
         <v>12</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G52" s="13" t="s">
         <v>42</v>
@@ -2958,7 +2958,7 @@
         <v>12</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G53" s="13" t="s">
         <v>43</v>
@@ -2982,7 +2982,7 @@
         <v>33</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>44</v>
@@ -2994,7 +2994,7 @@
         <v>25</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>27</v>
@@ -3006,10 +3006,10 @@
         <v>0.65</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G55" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H55" s="10"/>
     </row>
@@ -3030,10 +3030,10 @@
         <v>0.4</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H56" s="10"/>
     </row>
@@ -3054,10 +3054,10 @@
         <v>396</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H57" s="10"/>
     </row>
@@ -3075,10 +3075,10 @@
         <v>55</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G58" s="13" t="s">
         <v>46</v>
@@ -3099,10 +3099,10 @@
         <v>55</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>48</v>
@@ -3123,10 +3123,10 @@
         <v>55</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>47</v>
@@ -3147,10 +3147,10 @@
         <v>55</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>49</v>
@@ -3171,13 +3171,13 @@
         <v>55</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H62" s="10"/>
     </row>
@@ -3192,30 +3192,27 @@
         <v>31</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E63" s="2">
         <v>100</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H63" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3230,12 +3227,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3264,52 +3264,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+        <v>81</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3321,11 +3321,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3344,72 +3344,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3421,13 +3421,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3435,13 +3435,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3451,13 +3451,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3467,13 +3467,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3481,15 +3481,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="B15" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3497,13 +3497,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3550,7 +3550,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>42</v>
@@ -3574,7 +3574,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>43</v>
@@ -3598,7 +3598,7 @@
         <v>60</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>44</v>
@@ -3610,7 +3610,7 @@
         <v>25</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>27</v>
@@ -3622,10 +3622,10 @@
         <v>0.25</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H21" s="10"/>
     </row>
@@ -3646,10 +3646,10 @@
         <v>0.12</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H22" s="10"/>
     </row>
@@ -3670,10 +3670,10 @@
         <v>438</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H23" s="10"/>
     </row>
@@ -3691,10 +3691,10 @@
         <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>46</v>
@@ -3715,10 +3715,10 @@
         <v>55</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>48</v>
@@ -3739,10 +3739,10 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>47</v>
@@ -3763,10 +3763,10 @@
         <v>55</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>49</v>
@@ -3777,13 +3777,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3795,15 +3795,15 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H29" s="9"/>
     </row>
@@ -3811,15 +3811,15 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
+      <c r="B30" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
       <c r="G30" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3827,13 +3827,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="B31" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3880,7 +3880,7 @@
         <v>21</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>42</v>
@@ -3904,7 +3904,7 @@
         <v>33</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>43</v>
@@ -3928,7 +3928,7 @@
         <v>68</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>44</v>
@@ -3940,7 +3940,7 @@
         <v>25</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>27</v>
@@ -3952,10 +3952,10 @@
         <v>0.49</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H36" s="10"/>
     </row>
@@ -3976,10 +3976,10 @@
         <v>0.19</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H37" s="10"/>
     </row>
@@ -4000,10 +4000,10 @@
         <v>534</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H38" s="10"/>
     </row>
@@ -4021,10 +4021,10 @@
         <v>55</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>46</v>
@@ -4045,10 +4045,10 @@
         <v>55</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>48</v>
@@ -4069,10 +4069,10 @@
         <v>55</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>47</v>
@@ -4093,10 +4093,10 @@
         <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>49</v>
@@ -4107,13 +4107,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4125,15 +4125,15 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
+      <c r="B44" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
       <c r="G44" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H44" s="9"/>
     </row>
@@ -4141,15 +4141,15 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
+      <c r="B45" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
       <c r="G45" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -4157,13 +4157,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
+      <c r="B46" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4210,7 +4210,7 @@
         <v>33</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G48" s="13" t="s">
         <v>42</v>
@@ -4234,7 +4234,7 @@
         <v>51</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G49" s="13" t="s">
         <v>43</v>
@@ -4258,7 +4258,7 @@
         <v>75</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G50" s="13" t="s">
         <v>44</v>
@@ -4270,7 +4270,7 @@
         <v>25</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>27</v>
@@ -4282,10 +4282,10 @@
         <v>0.73</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H51" s="10"/>
     </row>
@@ -4306,10 +4306,10 @@
         <v>0.25</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H52" s="10"/>
     </row>
@@ -4330,10 +4330,10 @@
         <v>600</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H53" s="10"/>
     </row>
@@ -4351,10 +4351,10 @@
         <v>55</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>46</v>
@@ -4375,10 +4375,10 @@
         <v>55</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>48</v>
@@ -4399,10 +4399,10 @@
         <v>55</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>47</v>
@@ -4423,10 +4423,10 @@
         <v>55</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>49</v>
@@ -4435,15 +4435,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4458,12 +4455,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4492,52 +4492,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="20"/>
+      <c r="A2" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F2" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+        <v>110</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4549,11 +4549,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4572,72 +4572,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4663,15 +4663,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="9" t="s">
         <v>127</v>
-      </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="9" t="s">
-        <v>128</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4679,13 +4679,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4695,13 +4695,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4709,15 +4709,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="B15" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4725,13 +4725,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="B16" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4778,10 +4778,10 @@
         <v>520</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -4799,13 +4799,13 @@
         <v>55</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="11" t="s">
-        <v>70</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -4823,13 +4823,13 @@
         <v>55</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H20" s="10"/>
     </row>
@@ -4837,13 +4837,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4855,15 +4855,15 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="B22" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -4871,13 +4871,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="B23" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4924,10 +4924,10 @@
         <v>520</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="H25" s="10"/>
     </row>
@@ -4942,13 +4942,13 @@
         <v>31</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26" s="2">
         <v>1</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>47</v>
@@ -4972,7 +4972,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>48</v>
@@ -4993,13 +4993,13 @@
         <v>55</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -5020,10 +5020,10 @@
         <v>1</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -5041,13 +5041,13 @@
         <v>55</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H30" s="10"/>
     </row>
@@ -5068,15 +5068,29 @@
         <v>1</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H31" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -5087,20 +5101,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Added a heart driver damper to prevent craziness that has been observed to hose the baroreceptors. Updated COPD parameters.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55A49B3-CCC5-4E90-BE65-13CB8D2EA46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E4876F5-A718-4846-9921-97E53009F86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25710" yWindow="2040" windowWidth="29130" windowHeight="27735" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25290" yWindow="5175" windowWidth="27375" windowHeight="24210" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -611,37 +611,11 @@
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
   "Mode": "ContinuousMandatoryVentilation", 
   "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.42 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.1, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 42.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 17, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.28 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
   "InspiratoryPressure": { "ScalarPressure": { "Value": 14.5, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 12, "Unit": "1/min" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "ContinuousMandatoryVentilation", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 23.5, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
   }}
 }</t>
   </si>
@@ -681,6 +655,32 @@
   </si>
   <si>
     <t>VT (measured)</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 25, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 7, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "ContinuousMandatoryVentilation", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.42 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.1, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 43, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 17, "Unit": "1/min" } }
+  }}
+}</t>
   </si>
 </sst>
 </file>
@@ -888,15 +888,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -907,6 +898,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1315,52 +1315,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1372,11 +1372,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1395,72 +1395,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1472,13 +1472,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1488,13 +1488,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1502,29 +1502,29 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9" t="s">
         <v>114</v>
       </c>
       <c r="H13" s="9"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1640,10 +1640,10 @@
         <v>55</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>76</v>
@@ -1667,7 +1667,7 @@
         <v>0.05</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>82</v>
@@ -1694,7 +1694,7 @@
         <v>86</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H21" s="10"/>
     </row>
@@ -1712,10 +1712,10 @@
         <v>55</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>46</v>
@@ -1739,7 +1739,7 @@
         <v>75</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>48</v>
@@ -1763,7 +1763,7 @@
         <v>45</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>47</v>
@@ -1787,7 +1787,7 @@
         <v>0.95</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>49</v>
@@ -1808,10 +1808,10 @@
         <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>85</v>
@@ -1844,12 +1844,11 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1858,11 +1857,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1892,52 +1892,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1949,11 +1949,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1972,72 +1972,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2063,13 +2063,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2079,13 +2079,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2095,13 +2095,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2109,13 +2109,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>115</v>
       </c>
@@ -2125,13 +2125,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2301,7 +2301,7 @@
         <v>86</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H23" s="10"/>
     </row>
@@ -2453,13 +2453,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2471,13 +2471,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2487,13 +2487,13 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
       <c r="G32" s="9" t="s">
         <v>116</v>
       </c>
@@ -2503,13 +2503,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2679,7 +2679,7 @@
         <v>86</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H40" s="10"/>
     </row>
@@ -2831,13 +2831,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="18"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2849,13 +2849,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="19" t="s">
+      <c r="B48" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-      <c r="F48" s="19"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
       <c r="G48" s="9" t="s">
         <v>77</v>
       </c>
@@ -2865,13 +2865,13 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
+      <c r="B49" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
       <c r="G49" s="9" t="s">
         <v>117</v>
       </c>
@@ -2881,13 +2881,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -3057,7 +3057,7 @@
         <v>86</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H57" s="10"/>
     </row>
@@ -3207,12 +3207,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3227,15 +3230,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3264,52 +3264,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3321,11 +3321,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3344,72 +3344,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3421,13 +3421,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3435,13 +3435,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3451,13 +3451,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3467,13 +3467,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3481,13 +3481,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="B15" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>137</v>
       </c>
@@ -3497,13 +3497,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3571,7 +3571,7 @@
         <v>28</v>
       </c>
       <c r="E19" s="2">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>89</v>
@@ -3619,7 +3619,7 @@
         <v>28</v>
       </c>
       <c r="E21" s="2">
-        <v>0.25</v>
+        <v>0.37</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>91</v>
@@ -3673,7 +3673,7 @@
         <v>86</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H23" s="10"/>
     </row>
@@ -3777,13 +3777,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3795,13 +3795,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="9" t="s">
         <v>78</v>
       </c>
@@ -3811,13 +3811,13 @@
       <c r="A30" s="8">
         <v>2</v>
       </c>
-      <c r="B30" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
+      <c r="B30" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="9" t="s">
         <v>118</v>
       </c>
@@ -3827,13 +3827,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3877,7 +3877,7 @@
         <v>28</v>
       </c>
       <c r="E33" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>90</v>
@@ -3901,7 +3901,7 @@
         <v>28</v>
       </c>
       <c r="E34" s="2">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F34" s="11" t="s">
         <v>89</v>
@@ -4003,7 +4003,7 @@
         <v>86</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H38" s="10"/>
     </row>
@@ -4107,13 +4107,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4125,13 +4125,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
       <c r="G44" s="9" t="s">
         <v>79</v>
       </c>
@@ -4141,13 +4141,13 @@
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
+      <c r="B45" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" s="26"/>
+      <c r="D45" s="26"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="27"/>
       <c r="G45" s="9" t="s">
         <v>136</v>
       </c>
@@ -4157,13 +4157,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="B46" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4207,7 +4207,7 @@
         <v>28</v>
       </c>
       <c r="E48" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F48" s="11" t="s">
         <v>90</v>
@@ -4333,7 +4333,7 @@
         <v>86</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H53" s="10"/>
     </row>
@@ -4435,12 +4435,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4455,15 +4458,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4492,52 +4492,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4549,11 +4549,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4572,72 +4572,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4663,13 +4663,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>127</v>
       </c>
@@ -4679,13 +4679,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4695,13 +4695,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4709,13 +4709,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>119</v>
       </c>
@@ -4725,13 +4725,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4781,7 +4781,7 @@
         <v>69</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -4837,13 +4837,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4855,13 +4855,13 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
       <c r="G22" s="9" t="s">
         <v>125</v>
       </c>
@@ -4871,13 +4871,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4927,7 +4927,7 @@
         <v>69</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H25" s="10"/>
     </row>
@@ -5077,20 +5077,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -5101,6 +5087,20 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Tweak severe COPD shunting to match updated validation.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA299CB6-674D-4A27-8FF5-99BD7932766C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59CE000-7D91-425F-B039-A3E80FE1EC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28935" yWindow="3225" windowWidth="27375" windowHeight="26790" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28275" yWindow="4215" windowWidth="22065" windowHeight="23445" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -888,6 +888,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -898,15 +907,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1315,52 +1315,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1372,11 +1372,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1395,72 +1395,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1472,13 +1472,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1488,13 +1488,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1502,13 +1502,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
         <v>113</v>
       </c>
@@ -1518,13 +1518,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1844,11 +1844,12 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1857,12 +1858,11 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1892,52 +1892,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="226.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1949,11 +1949,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1972,72 +1972,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2063,13 +2063,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2079,13 +2079,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2095,13 +2095,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2109,13 +2109,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>114</v>
       </c>
@@ -2125,13 +2125,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2453,13 +2453,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2471,13 +2471,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2487,13 +2487,13 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
       <c r="G32" s="9" t="s">
         <v>115</v>
       </c>
@@ -2503,13 +2503,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2831,13 +2831,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2849,13 +2849,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
       <c r="G48" s="9" t="s">
         <v>77</v>
       </c>
@@ -2865,13 +2865,13 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="22" t="s">
+      <c r="B49" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="C49" s="22"/>
-      <c r="D49" s="22"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
       <c r="G49" s="9" t="s">
         <v>116</v>
       </c>
@@ -2881,13 +2881,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="22" t="s">
+      <c r="B50" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C50" s="22"/>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -3207,15 +3207,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3230,12 +3227,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3264,52 +3264,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="284.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3321,11 +3321,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3344,72 +3344,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3421,13 +3421,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3435,13 +3435,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3451,13 +3451,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3467,13 +3467,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3481,13 +3481,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>142</v>
       </c>
@@ -3497,13 +3497,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3777,13 +3777,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3795,13 +3795,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="9" t="s">
         <v>78</v>
       </c>
@@ -3827,13 +3827,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -4107,13 +4107,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4125,13 +4125,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
       <c r="G44" s="9" t="s">
         <v>79</v>
       </c>
@@ -4157,13 +4157,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4303,7 +4303,7 @@
         <v>28</v>
       </c>
       <c r="E52" s="2">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>92</v>
@@ -4435,15 +4435,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4458,12 +4455,15 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4492,52 +4492,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="20"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4549,11 +4549,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4572,72 +4572,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="23" t="s">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="23" t="s">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="23" t="s">
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="23" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4663,13 +4663,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>126</v>
       </c>
@@ -4679,13 +4679,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4695,13 +4695,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4709,13 +4709,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
         <v>118</v>
       </c>
@@ -4725,13 +4725,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4837,13 +4837,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4855,13 +4855,13 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="9" t="s">
         <v>124</v>
       </c>
@@ -4871,13 +4871,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -5077,6 +5077,20 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -5087,20 +5101,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Fixed a couple citations.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD190F7C-13DE-4B9A-B9EF-1D2DBCDD5B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28622775-04F4-48BB-AFAB-0B7ECD02F8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="7560" windowWidth="31935" windowHeight="17025" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -661,10 +661,10 @@
   <si>
     <t>A healthy male patient with a predicted body weight of 60 kg is mechanically ventilated.  These are the data sources:
  - Resistance: Inspiratory resistance (Rinsp) is assumed equal to expiratory resistance (Rexp), taken from Arnal et al @cite arnal2018parameters (Table 9).
- - Compliance: Taken from Arnal et al arnal2018parameters (Table 3). 
+ - Compliance: Taken from Arnal et al @cite arnal2018parameters (Table 3). 
  - Dead space:  Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care page 63 @cite kacmarek2016egan.
  - Shunt:  Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care page 68 @cite kacmarek2016egan.
- - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et alv @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
+ - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
  - Blood Gas Values: Standard healthy values taken from the Kacmarek et al Fundamentals of Respiratory Care @cite kacmarek2016egan.</t>
   </si>
   <si>
@@ -673,7 +673,7 @@
  - Compliance: All compliances were taken from Maj et al @cite maj2023ventilatory (Table 1) derived as tidal volume (ie, mL/kg x PBW calcualted with ARDS equation for males) divided by driving pressure. Mild ARDS was mean minus 1  standard deviatio; moderate ARDS was the mean value; severe ARDS was mean plus 1  standard deviation. 
  - Dead space:  VD/VT values were taken from Maj et al @cite maj2023ventilatory (Table 2). 
  - Shunt:  Values for QS/QT were a compromise between Maj et al @cite maj2023ventilatory (Table 2, venous admixture) and Torres et al @cite torres1989ventilation (Table 3) to give realistic PO2 results for the simulated ventilator settings.    
- - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et alv @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
+ - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
  - Blood Gas Values: Expected blood gas value for outputs of Pulse simulator were taken from the most complete source: Arnal et al @cite arnal2018parameters (Table 2). FiO2 values for moderate and severe ARDS were adjusted upward to give the expected P/F ratios for the given PaO2 ranges. Expected values for SpO2 were calculated from PaO2 using the equation from Gadrey et al @cite gadrey2019imputation.</t>
   </si>
   <si>
@@ -682,7 +682,7 @@
  - Compliance: All compliances were taken from Arnal et al @cite arnal2018parameters (Table 3). Mild COPD was approximately the mean value (so as to be higher than normal); moderate COPD was the average of the mean and the high end of the range (60,75), and severe COPD was the highest value of the range.
  - Dead space:  VD/VT values were taken from Farah et al @cite farah2009can (Table 1). Mild COPD was mean minus 1 standard deviation; moderate COPD was the mean value; severe COPD was mean plus 2 standard deviations. 
  - Shunt: QS/QT values were taken from Torres et al @cite torres1989ventilation (Table 3). Mild COPD was mean minus 2 standard deviations; moderate COPD was the mean value; for severe COPD, values for FiO2 and PaO2 were taken from Arnal et al @cite arnal2018parameters (Table 2) and used with various prediction equations for iso-shunt lines to get a match at about PaO2 = 69, FiO2 = 0.4 and shunt = 0.20 .
- - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et alv @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
+ - Ventilator Settings: All ventilator settings were takeng from Arnal et al @cite arnal2018parameters (Table 2) for a male patient aged 73 years and predicted body weight of 60 kg. Note that the mode for simulation is PC-CMV, which is equivalent to the mode used by Arnal et @cite arnal2018parameters for passive pateints. Equivalent settings for tidal volume, rate, and inspiratory time can be used for volume control simulations.
  - Blood Gas Values: Expected blood gas value for outputs of Pulse simulator were taken from the most complete source: Arnal et al @cite arnal2018parameters (Table 2). Expected values for SpO2 were calculated from PaO2 using the equation from Gadrey et al @cite gadrey2019imputation.</t>
   </si>
 </sst>
@@ -891,15 +891,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -910,6 +901,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1318,50 +1318,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1373,11 +1373,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1396,72 +1396,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1473,13 +1473,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1489,13 +1489,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1503,13 +1503,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9" t="s">
         <v>112</v>
       </c>
@@ -1519,13 +1519,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1845,12 +1845,11 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -1859,11 +1858,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1893,50 +1893,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="241.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1948,11 +1948,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1971,72 +1971,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2062,13 +2062,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>63</v>
       </c>
@@ -2078,13 +2078,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2094,13 +2094,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2108,13 +2108,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>113</v>
       </c>
@@ -2124,13 +2124,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2452,13 +2452,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2470,13 +2470,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2486,13 +2486,13 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
       <c r="G32" s="9" t="s">
         <v>114</v>
       </c>
@@ -2502,13 +2502,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2830,13 +2830,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="18"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2848,13 +2848,13 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="19" t="s">
+      <c r="B48" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-      <c r="F48" s="19"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
       <c r="G48" s="9" t="s">
         <v>77</v>
       </c>
@@ -2864,13 +2864,13 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="19" t="s">
+      <c r="B49" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
       <c r="G49" s="9" t="s">
         <v>115</v>
       </c>
@@ -2880,13 +2880,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -3206,12 +3206,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -3226,15 +3229,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3263,50 +3263,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="267" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3318,11 +3318,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3341,72 +3341,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3418,13 +3418,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3432,13 +3432,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>64</v>
       </c>
@@ -3448,13 +3448,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3464,13 +3464,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3478,13 +3478,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>141</v>
       </c>
@@ -3494,13 +3494,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3774,13 +3774,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3792,13 +3792,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="9" t="s">
         <v>78</v>
       </c>
@@ -3824,13 +3824,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -4104,13 +4104,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4122,13 +4122,13 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
       <c r="G44" s="9" t="s">
         <v>79</v>
       </c>
@@ -4154,13 +4154,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="B46" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4432,12 +4432,15 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B43:F43"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
@@ -4452,15 +4455,12 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4489,50 +4489,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4544,11 +4544,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4567,72 +4567,72 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21" t="s">
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21" t="s">
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4658,13 +4658,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="9" t="s">
         <v>125</v>
       </c>
@@ -4674,13 +4674,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4690,13 +4690,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4704,13 +4704,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="9" t="s">
         <v>117</v>
       </c>
@@ -4720,13 +4720,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4832,13 +4832,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4850,13 +4850,13 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
       <c r="G22" s="9" t="s">
         <v>123</v>
       </c>
@@ -4866,13 +4866,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -5072,20 +5072,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
@@ -5096,6 +5082,20 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>